<commit_message>
Add_script, TextPrinter and the commands Duel demo generation
</commit_message>
<xml_diff>
--- a/ContentLibraryService/AssetsDatabase.xlsx
+++ b/ContentLibraryService/AssetsDatabase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyStuffs\BU\Projects\T2G\ContentLibraryService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC83795-D445-4385-897F-368090B43619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70013E5A-450D-4A00-B91E-D4DE547F7820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6818" yWindow="8198" windowWidth="21600" windowHeight="9472" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
+    <workbookView xWindow="2805" yWindow="2175" windowWidth="21600" windowHeight="12128" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
   </bookViews>
   <sheets>
     <sheet name="AssetsDatabase" sheetId="1" r:id="rId1"/>
@@ -196,9 +196,6 @@
     <t>Packages/Cameras/ObserveCamera.unitypackage,Prefabs/Cameras/ObserveCamera.prefab</t>
   </si>
   <si>
-    <t>Packages/Natual/Sky.unitypackage,Prefabs/Natual/SKy/Sky Dome.prefab</t>
-  </si>
-  <si>
     <t>Packages/Natual/Sun.unitypackage,Prefabs/Natual/Sun.prefab</t>
   </si>
   <si>
@@ -284,6 +281,9 @@
   </si>
   <si>
     <t>Packages/Knight/Knight.unitypackage,Prefabs/Knight/Knight.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Natual/Sky.unitypackage,Prefabs/Natual/Sky/Sky Dome.prefab</t>
   </si>
 </sst>
 </file>
@@ -1401,7 +1401,7 @@
         <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
@@ -1415,7 +1415,7 @@
         <v>29</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1429,133 +1429,133 @@
         <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
         <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
         <v>29</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
         <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C25" t="s">
         <v>29</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
         <v>29</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C27" t="s">
         <v>29</v>
       </c>
       <c r="D27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" t="s">
         <v>29</v>
       </c>
       <c r="D28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C29" t="s">
         <v>29</v>
       </c>
       <c r="D29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build structure support, Add script support
</commit_message>
<xml_diff>
--- a/ContentLibraryService/AssetsDatabase.xlsx
+++ b/ContentLibraryService/AssetsDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyStuffs\BU\Projects\T2G\ContentLibraryService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70013E5A-450D-4A00-B91E-D4DE547F7820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE5B189-7591-4B32-8125-B5D1BD6D3694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2805" yWindow="2175" windowWidth="21600" windowHeight="12128" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="106">
   <si>
     <t>name</t>
   </si>
@@ -284,6 +284,60 @@
   </si>
   <si>
     <t>Packages/Natual/Sky.unitypackage,Prefabs/Natual/Sky/Sky Dome.prefab</t>
+  </si>
+  <si>
+    <t>Tree1</t>
+  </si>
+  <si>
+    <t>Tree2</t>
+  </si>
+  <si>
+    <t>Tree3</t>
+  </si>
+  <si>
+    <t>Tree4</t>
+  </si>
+  <si>
+    <t>Tree5</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree1.unitypackage,Prefabs/Trees/Tree1.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree2.unitypackage,Prefabs/Trees/Tree2.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree3.unitypackage,Prefabs/Trees/Tree3.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree4.unitypackage,Prefabs/Trees/Tree4.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree5.unitypackage,Prefabs/Trees/Tree5.prefab</t>
+  </si>
+  <si>
+    <t>Tree 1</t>
+  </si>
+  <si>
+    <t>Tree 2</t>
+  </si>
+  <si>
+    <t>Tree 3</t>
+  </si>
+  <si>
+    <t>Tree6</t>
+  </si>
+  <si>
+    <t>Tree 6 small</t>
+  </si>
+  <si>
+    <t>Tree 5 small</t>
+  </si>
+  <si>
+    <t>Tree 4 Middle</t>
+  </si>
+  <si>
+    <t>Packages/Trees/Tree6.unitypackage,Prefabs/Trees/Tree6.prefab</t>
   </si>
 </sst>
 </file>
@@ -1144,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9730564A-27F9-4669-AA8A-3D3510692C17}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.53125" customWidth="1"/>
@@ -1558,6 +1612,90 @@
         <v>86</v>
       </c>
     </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" t="s">
+        <v>29</v>
+      </c>
+      <c r="D33" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" t="s">
+        <v>103</v>
+      </c>
+      <c r="C34" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>101</v>
+      </c>
+      <c r="B35" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" t="s">
+        <v>29</v>
+      </c>
+      <c r="D35" t="s">
+        <v>105</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Using async executions and commands to improve the system quality. Fixed bugs
</commit_message>
<xml_diff>
--- a/ContentLibraryService/AssetsDatabase.xlsx
+++ b/ContentLibraryService/AssetsDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyStuffs\BU\Projects\T2G\ContentLibraryService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE5B189-7591-4B32-8125-B5D1BD6D3694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73819FA2-4BEE-45BF-A8BF-6DAF5CB4D861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2805" yWindow="2175" windowWidth="21600" windowHeight="12128" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>default</t>
   </si>
   <si>
-    <t>Prefabs/Primitives/cube.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
     <t>capsule</t>
   </si>
   <si>
@@ -49,9 +46,6 @@
     <t>prefab</t>
   </si>
   <si>
-    <t>Prefabs/Primitives/capsule.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
     <t>cube</t>
   </si>
   <si>
@@ -76,18 +70,6 @@
     <t>primitive sphere</t>
   </si>
   <si>
-    <t>Prefabs/Primitives/cylinder.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
-    <t>Prefabs/Primitives/plane.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
-    <t>Prefabs/Primitives/quade.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
-    <t>Prefabs/Primitives/sphere.prefab,Scripts/ObjectInterface.cs</t>
-  </si>
-  <si>
     <t>spin controller</t>
   </si>
   <si>
@@ -259,24 +241,6 @@
     <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_AK.prefab</t>
   </si>
   <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_G36.prefab</t>
-  </si>
-  <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_L85.prefab</t>
-  </si>
-  <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_M4.prefab</t>
-  </si>
-  <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_MP5.prefab</t>
-  </si>
-  <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_Scar.prefab</t>
-  </si>
-  <si>
-    <t>Packages/Guns/Gun_AK.unitypackage,Prefabs/Guns/Gun_AK/Gun_Type97.prefab</t>
-  </si>
-  <si>
     <t>Packages/UI/SimpleUI.unitypackage,Prefabs/SimpleUI/SimpleUI.prefab</t>
   </si>
   <si>
@@ -338,6 +302,42 @@
   </si>
   <si>
     <t>Packages/Trees/Tree6.unitypackage,Prefabs/Trees/Tree6.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_G36.unitypackage,Prefabs/Guns/Gun_G36/Gun_G36.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_L85.unitypackage,Prefabs/Guns/Gun_L85/Gun_L85.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_M4.unitypackage,Prefabs/Guns/Gun_M4/Gun_M4.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_MP5.unitypackage,Prefabs/Guns/Gun_MP5/Gun_MP5.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_Type97.unitypackage,Prefabs/Guns/Gun_Type97/Gun_Type97.prefab</t>
+  </si>
+  <si>
+    <t>Packages/Guns/Gun_Scar.unitypackage,Prefabs/Guns/Gun_Scar/Gun_Scar.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/cube.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/capsule.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/cylinder.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/plane.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/quade.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Primitives/sphere.prefab</t>
   </si>
 </sst>
 </file>
@@ -821,8 +821,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1207,16 +1208,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1231,469 +1232,469 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
         <v>38</v>
       </c>
-      <c r="B17" t="s">
-        <v>44</v>
-      </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D23" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C25" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C27" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C29" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="B31" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C32" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B33" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="C33" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D35" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attach, Dettach, MakePrefab instructions. Overwrite script when importing Fixed timeout no restored issue.
</commit_message>
<xml_diff>
--- a/ContentLibraryService/AssetsDatabase.xlsx
+++ b/ContentLibraryService/AssetsDatabase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyStuffs\BU\Projects\T2G\ContentLibraryService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73819FA2-4BEE-45BF-A8BF-6DAF5CB4D861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD20D9A-86D8-4159-9F86-A26F85C2D4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2805" yWindow="2175" windowWidth="21600" windowHeight="12128" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
+    <workbookView xWindow="4043" yWindow="4043" windowWidth="21599" windowHeight="12682" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
   </bookViews>
   <sheets>
     <sheet name="AssetsDatabase" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="122">
   <si>
     <t>name</t>
   </si>
@@ -338,6 +338,54 @@
   </si>
   <si>
     <t>Prefabs/Primitives/sphere.prefab</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>PerspectiveCamera</t>
+  </si>
+  <si>
+    <t>OrthognalCamera</t>
+  </si>
+  <si>
+    <t>DirectionalLight</t>
+  </si>
+  <si>
+    <t>PointLight</t>
+  </si>
+  <si>
+    <t>SpotLight</t>
+  </si>
+  <si>
+    <t>Directional light</t>
+  </si>
+  <si>
+    <t>Point light</t>
+  </si>
+  <si>
+    <t>Spot light</t>
+  </si>
+  <si>
+    <t>Orthognal orthorgraphics camera</t>
+  </si>
+  <si>
+    <t>Prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Cameras/Camera.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Cameras/OrthognalCamera.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Lights/DirectionalLight.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Lights/PointLight.prefab</t>
+  </si>
+  <si>
+    <t>Prefabs/Lights/SpotLight.prefab</t>
   </si>
 </sst>
 </file>
@@ -1199,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9730564A-27F9-4669-AA8A-3D3510692C17}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.53125" customWidth="1"/>
@@ -1697,6 +1745,76 @@
         <v>93</v>
       </c>
     </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" t="s">
+        <v>116</v>
+      </c>
+      <c r="D36" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" t="s">
+        <v>115</v>
+      </c>
+      <c r="C37" t="s">
+        <v>116</v>
+      </c>
+      <c r="D37" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" t="s">
+        <v>112</v>
+      </c>
+      <c r="C38" t="s">
+        <v>116</v>
+      </c>
+      <c r="D38" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" t="s">
+        <v>113</v>
+      </c>
+      <c r="C39" t="s">
+        <v>116</v>
+      </c>
+      <c r="D39" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" t="s">
+        <v>116</v>
+      </c>
+      <c r="D40" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ContentLibrary database update and add_behaviour update
</commit_message>
<xml_diff>
--- a/ContentLibraryService/AssetsDatabase.xlsx
+++ b/ContentLibraryService/AssetsDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyStuffs\BU\Projects\T2G\ContentLibraryService\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD20D9A-86D8-4159-9F86-A26F85C2D4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF86AF2-8EC1-4E32-8E9A-3937894AB2E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4043" yWindow="4043" windowWidth="21599" windowHeight="12682" xr2:uid="{31D62863-9DD9-44FB-B2E4-58795221A0F9}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="124">
   <si>
     <t>name</t>
   </si>
@@ -370,9 +370,6 @@
     <t>Orthognal orthorgraphics camera</t>
   </si>
   <si>
-    <t>Prefab</t>
-  </si>
-  <si>
     <t>Prefabs/Cameras/Camera.prefab</t>
   </si>
   <si>
@@ -386,6 +383,15 @@
   </si>
   <si>
     <t>Prefabs/Lights/SpotLight.prefab</t>
+  </si>
+  <si>
+    <t>VolumeSpawner</t>
+  </si>
+  <si>
+    <t>Volume spawner</t>
+  </si>
+  <si>
+    <t>Packages/VolumeSpawner.unitypackage,Prefabs/VolumeSpawner.prefab</t>
   </si>
 </sst>
 </file>
@@ -1247,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9730564A-27F9-4669-AA8A-3D3510692C17}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.53125" customWidth="1"/>
@@ -1753,10 +1759,10 @@
         <v>106</v>
       </c>
       <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" t="s">
         <v>116</v>
-      </c>
-      <c r="D36" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
@@ -1767,10 +1773,10 @@
         <v>115</v>
       </c>
       <c r="C37" t="s">
-        <v>116</v>
+        <v>7</v>
       </c>
       <c r="D37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
@@ -1781,10 +1787,10 @@
         <v>112</v>
       </c>
       <c r="C38" t="s">
-        <v>116</v>
+        <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
@@ -1795,10 +1801,10 @@
         <v>113</v>
       </c>
       <c r="C39" t="s">
-        <v>116</v>
+        <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
@@ -1809,10 +1815,24 @@
         <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>116</v>
+        <v>7</v>
       </c>
       <c r="D40" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
         <v>121</v>
+      </c>
+      <c r="B41" t="s">
+        <v>122</v>
+      </c>
+      <c r="C41" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>